<commit_message>
feat: sincronizar planilhas de sinais, logs e novos estudos de metodos aprovados
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-08-28.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-08-28.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/21df80ec97692de0/Documentos/GitHub/ARKAD_PROD/metodos_aprovados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="11_2B59D18754CA3B29CB593C115950D8F275D7EF04" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA5A0833-3317-47E3-BDDA-47215A94C8B3}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="11_2B59D18754CA3B29CB593C115950D8F275D7EF04" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A4DB174-EA5D-48EC-A370-F06A622A57AD}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -278,7 +278,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1132,6 +1132,13 @@
       <c r="K13" t="s">
         <v>26</v>
       </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+      <c r="M13">
+        <f t="shared" si="0"/>
+        <v>6.8928571428571422E-2</v>
+      </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -1166,6 +1173,13 @@
       </c>
       <c r="K14" t="s">
         <v>26</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
+      <c r="M14">
+        <f t="shared" si="0"/>
+        <v>7.4230769230769225E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>